<commit_message>
feat: atualizar visitantes e separar cultos de domingo
</commit_message>
<xml_diff>
--- a/visitantes-2.0.xlsx
+++ b/visitantes-2.0.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4283,6 +4283,1358 @@
         <v>46205</v>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>5714</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>26/07/2026 20:50</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Marcos de Jesud</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>(11) 95429-8069</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>5712</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>26/07/2026 20:45</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Maria eliene</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>(11) 97730-7470</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>5713</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>26/07/2026 20:45</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Cristiano Ribeiro</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>(11) 95104-2847</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>5711</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>26/07/2026 20:44</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Mariane</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Passou na Frente</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>(11) 94716-3592</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>5708</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>26/07/2026 20:43</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Barbara</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>(11) 95811-0696</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>5709</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>26/07/2026 20:43</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Rodrigo de Almeida Ramos</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>(11) 97992-8653</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>5710</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>26/07/2026 20:43</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Caroline</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Passou na Frente</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>(11) 94728-9494</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>5706</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>26/07/2026 20:42</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Paulo Henrique</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>(11) 99633-3162</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>5707</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>26/07/2026 20:42</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Simone</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>(11) 95217-4598</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>5705</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>26/07/2026 12:26</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Beatriz</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>(11) 96240-3769</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>5703</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>26/07/2026 12:25</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Ormis Daniel Lagar Videaux</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>(11) 98420-4814</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>5704</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>26/07/2026 12:25</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Débora Cristina dos Santos Alves</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>(11) 98761-6277</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>5702</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>26/07/2026 12:24</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Wanessa alves</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>(11) 96157-0949</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>5694</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>21/07/2026 22:21</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Layana</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>(11) 97736-0498</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>5691</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>21/07/2026 22:18</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Damares</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>(11) 94860-4612</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>5692</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>21/07/2026 22:18</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Edilaine Firminino modesto da Silva</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Passou na Frente</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>(11) 99222-9671</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Café de boas vindas</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>5693</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>21/07/2026 22:18</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Daniele Oliveira</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>(11) 97075-6188</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>5688</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>21/07/2026 22:17</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Bianca Fernandes</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>(11) 95989-7085</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>5689</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>21/07/2026 22:17</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Branda heloise</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>(11) 97725-7808</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>5690</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>21/07/2026 22:17</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Cicero</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>(11) 94899-4186</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>5687</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>21/07/2026 22:16</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Juliana gallet</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>(11) 94897-2704</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>5685</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>21/07/2026 22:14</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Ester</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>(11) 98134-2017</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>5686</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>21/07/2026 22:14</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Sara Victoria</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Célula</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>(11) 93942-4160</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>5683</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>21/07/2026 22:13</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Matheus</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>(11) 95791-9407</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>5684</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>21/07/2026 22:13</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Shirley cicera</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>(11) 99232-0668</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>5682</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>21/07/2026 22:12</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Suene</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>(11) 95791-4263</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
feat: atualizar visitantes pós-26/07 e adicionar participação por culto
Inclui 36 novos visitantes (28/07–02/08/2026), passa a ler membros-2.0.xlsx
com member_count/children_count e adiciona KPIs e gráfico Chart.js de
membros × crianças por culto no painel.

Co-authored-by: Lucas Andrade Silva <LucasAndradeSilva@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/visitantes-2.0.xlsx
+++ b/visitantes-2.0.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J102"/>
+  <dimension ref="A1:J138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5635,6 +5635,1807 @@
         </is>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>5721</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>28/07/2026 20:00</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Daniele Alves</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>(11) 95432-1479</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>5722</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>28/07/2026 20:01</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Gabriel Silva</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>(11) 91938-7966</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>5725</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>28/07/2026 22:12</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Igor Rodrigues</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>(11) 98183-5820</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Amigo que teouxe</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>5726</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>28/07/2026 22:14</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Ana Beatriz de Sousa</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>(11) 99625-6915</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>5727</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>28/07/2026 22:14</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Arnold Santod</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>(11) 99012-9844</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>5728</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>28/07/2026 22:15</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Jonathan Oliveira</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>(11) 99012-9844</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Telefone é o do pai dele.
+Jonathan tem 13 anos</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>5729</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>28/07/2026 22:15</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Julia Martins</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>(11) 98100-6027</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>5733</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>30/07/2026 19:29</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Raquel</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>(11) 98605-3949</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>5734</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>30/07/2026 19:51</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Elisabete</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>(11) 99412-7883</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>5735</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>30/07/2026 19:53</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Maria Jose</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>(11) 95336-4809</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>5736</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>30/07/2026 22:02</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Graziela</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Passou na Frente</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>(11) 94843-7859</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>5737</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>30/07/2026 22:02</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Leticia Nunes</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>(11) 97529-7072</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>5738</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>30/07/2026 22:03</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Elaine Nunes</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>(11) 99916-1637</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>5739</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>30/07/2026 22:03</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Carolina Nunes</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>(11) 93440-2711</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>5740</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>30/07/2026 22:04</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Victor Pires</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>(11) 93019-0788</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>5741</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>30/07/2026 22:04</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Bianca</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>(11) 91147-1403</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>5773</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>01/08/2026 21:48</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>João pedro</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Célula</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>(11) 96070-8277</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Célula Fervorosos</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>5781</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>02/08/2026 10:00</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Maria das graças</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>(11) 94507-2092</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>5783</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>02/08/2026 10:20</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Guilherme Alencar</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>(11) 98789-2748</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>5784</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>02/08/2026 10:33</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Micheli Vanessa da Silva</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>(11) 97638-9250</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>5787</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>02/08/2026 12:37</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Diana mendes barbosa</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>(11) 93756-2825</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>5788</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>02/08/2026 12:37</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Sandy Silva</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>(11) 98945-6978</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Sem célula</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>5789</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>02/08/2026 12:37</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Guilherme</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>(11) 91059-1231</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>5790</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>02/08/2026 12:38</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Andressa hata</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>(11) 95279-4939</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Sem célula</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>5791</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>02/08/2026 12:38</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Rafaela da silva</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>(11) 95961-6095</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>5792</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>02/08/2026 12:40</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Lorena rodrigues Silva</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Célula</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>(11) 97682-2219</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>5793</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>02/08/2026 12:40</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Adriana Correia</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>(11) 99629-7486</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Sem célula</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>5794</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>02/08/2026 12:40</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Daniel fagner Lima</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>(11) 96809-7307</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>5795</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>02/08/2026 14:39</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Rafaela</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>(11) 95961-9065</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Café com os Pastores - primeira vez</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Culto Manhã</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>5799</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>02/08/2026 21:03</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Elaine Odete Oliveira</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Outras Redes Sociais</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>(11) 94254-1317</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>5800</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>02/08/2026 21:04</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Rafael Santos de Oliveira</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Masculino 👨</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>(15) 99178-8533</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>5801</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>02/08/2026 21:05</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Maria leiliane de Araújo Soares</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>(11) 96782-8784</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>5802</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>02/08/2026 21:05</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Lucy Cunha</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>(11) 98312-0810</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>5803</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>02/08/2026 21:05</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Elaine Ferreira</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Amigo/Familiar</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>(11) 98826-4220</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>5804</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>02/08/2026 21:07</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Jaqueline Martins</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>(11) 98707-1809</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Shalon</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>5805</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>02/08/2026 21:09</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Claudenice Santos bezerra</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Feminino 🚺</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Passou na Frente</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>(11) 95168-7960</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Culto Noite</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>

</xml_diff>